<commit_message>
Add 2019 exam papers, OCR results, images, and update questions and data
</commit_message>
<xml_diff>
--- a/정답표/정답표.xlsx
+++ b/정답표/정답표.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eboso\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eboso\Desktop\기말고사\security-study-app\정답표\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EC7A157-4AE6-40DA-B6BE-B844B32EC8F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9425278-5F20-4900-B717-E589BBDD72D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{79D6B732-5C55-4E7D-A9AF-6DF238744733}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{79D6B732-5C55-4E7D-A9AF-6DF238744733}"/>
   </bookViews>
   <sheets>
     <sheet name="2018" sheetId="1" r:id="rId1"/>
     <sheet name="2019" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="33">
   <si>
     <t>컴퓨터보안</t>
   </si>
@@ -121,7 +121,12 @@
     <t>1,2,3,4</t>
   </si>
   <si>
-    <t>유비쿼터스</t>
+    <t>유비쿼터스컴퓨팅개론</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>유비쿼터스컴퓨팅개론</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -314,10 +319,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -636,6 +641,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E35209E2-99BD-46C0-9861-50C8F6851C92}">
   <dimension ref="A1:AK10"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="19.25" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:37" ht="17.25" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -714,10 +722,10 @@
       </c>
     </row>
     <row r="3" spans="1:37" ht="17.25" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="8" t="s">
         <v>6</v>
       </c>
       <c r="C3">
@@ -827,8 +835,8 @@
       </c>
     </row>
     <row r="4" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A4" s="8"/>
-      <c r="B4" s="7"/>
+      <c r="A4" s="7"/>
+      <c r="B4" s="8"/>
       <c r="C4">
         <v>36</v>
       </c>
@@ -1415,7 +1423,7 @@
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C10">
         <v>2</v>
@@ -1537,6 +1545,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FFE4C3A-83AE-42BF-8F58-9A46633D3A63}">
   <dimension ref="A1:AK10"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="36.125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:37" ht="17.25" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -1615,10 +1626,10 @@
       </c>
     </row>
     <row r="3" spans="1:37" ht="17.25" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="8" t="s">
         <v>6</v>
       </c>
       <c r="C3">
@@ -1728,8 +1739,8 @@
       </c>
     </row>
     <row r="4" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A4" s="8"/>
-      <c r="B4" s="7"/>
+      <c r="A4" s="7"/>
+      <c r="B4" s="8"/>
       <c r="C4">
         <v>36</v>
       </c>

</xml_diff>